<commit_message>
Docs] Modify damage calculator
-노말 장비 궁극기 계산 오류 수정
</commit_message>
<xml_diff>
--- a/Project_Design/데미지 계산기.xlsx
+++ b/Project_Design/데미지 계산기.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wjdgn\OneDrive\문서\GitHub\Project_SkyPower\Project_Design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D88F718-F1CC-4690-9529-B8FC06250549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74544279-CC80-4D01-ADDA-B4189CFDBC4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B9A3E7C9-B38E-4C5D-B478-62826952F2F9}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="529" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="217">
   <si>
     <t>DPS</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1353,38 +1353,6 @@
         <charset val="129"/>
       </rPr>
       <t>성</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>루나</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>&lt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>클레아</t>
     </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -2081,7 +2049,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2134,7 +2102,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -2194,9 +2162,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2212,20 +2177,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2251,13 +2207,7 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2586,7 +2536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75CF228F-51F7-4050-917F-1EA0D0CDA272}">
-  <dimension ref="D2:AD42"/>
+  <dimension ref="D2:AD41"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="3" width="8.6640625" style="19"/>
@@ -2596,7 +2546,7 @@
     <col min="7" max="7" width="10.58203125" style="19" customWidth="1"/>
     <col min="8" max="8" width="11.5" style="19" customWidth="1"/>
     <col min="9" max="9" width="15.33203125" style="19" customWidth="1"/>
-    <col min="10" max="10" width="6.1640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.58203125" style="19" customWidth="1"/>
     <col min="11" max="11" width="10.25" style="19" customWidth="1"/>
     <col min="12" max="12" width="12.33203125" style="19" customWidth="1"/>
     <col min="13" max="13" width="6.83203125" style="19" bestFit="1" customWidth="1"/>
@@ -2622,8 +2572,8 @@
     <row r="3" spans="4:30" ht="14.5" thickBot="1"/>
     <row r="4" spans="4:30" ht="14.5" thickBot="1">
       <c r="W4" s="21"/>
-      <c r="X4" s="60" t="s">
-        <v>217</v>
+      <c r="X4" s="54" t="s">
+        <v>216</v>
       </c>
       <c r="Y4" s="21"/>
       <c r="Z4" s="21"/>
@@ -2637,7 +2587,7 @@
         <v>170</v>
       </c>
       <c r="W5" s="21"/>
-      <c r="X5" s="61" t="s">
+      <c r="X5" s="55" t="s">
         <v>131</v>
       </c>
       <c r="Y5" s="21"/>
@@ -2678,11 +2628,11 @@
       <c r="Q6" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="S6" s="57"/>
-      <c r="T6" s="58"/>
-      <c r="U6" s="58"/>
-      <c r="V6" s="58"/>
-      <c r="W6" s="58"/>
+      <c r="S6" s="35"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="23"/>
+      <c r="V6" s="23"/>
+      <c r="W6" s="23"/>
       <c r="X6" s="22" t="s">
         <v>180</v>
       </c>
@@ -2732,11 +2682,11 @@
       <c r="Q7" s="3">
         <v>10</v>
       </c>
-      <c r="S7" s="38"/>
+      <c r="S7" s="20"/>
       <c r="T7" s="18"/>
-      <c r="U7" s="59"/>
+      <c r="U7" s="53"/>
       <c r="V7" s="18"/>
-      <c r="W7" s="59"/>
+      <c r="W7" s="53"/>
       <c r="X7" s="29">
         <v>20</v>
       </c>
@@ -2786,11 +2736,11 @@
       <c r="Q8" s="3">
         <v>10</v>
       </c>
-      <c r="S8" s="38"/>
+      <c r="S8" s="20"/>
       <c r="T8" s="18"/>
-      <c r="U8" s="59"/>
+      <c r="U8" s="53"/>
       <c r="V8" s="18"/>
-      <c r="W8" s="59"/>
+      <c r="W8" s="53"/>
       <c r="X8" s="31">
         <v>20</v>
       </c>
@@ -2840,11 +2790,11 @@
       <c r="Q9" s="3">
         <v>10</v>
       </c>
-      <c r="S9" s="38"/>
+      <c r="S9" s="20"/>
       <c r="T9" s="18"/>
-      <c r="U9" s="59"/>
+      <c r="U9" s="53"/>
       <c r="V9" s="18"/>
-      <c r="W9" s="59"/>
+      <c r="W9" s="53"/>
       <c r="X9" s="31">
         <v>20</v>
       </c>
@@ -2892,11 +2842,11 @@
       <c r="Q10" s="3">
         <v>10</v>
       </c>
-      <c r="S10" s="38"/>
+      <c r="S10" s="20"/>
       <c r="T10" s="18"/>
-      <c r="U10" s="59"/>
+      <c r="U10" s="53"/>
       <c r="V10" s="18"/>
-      <c r="W10" s="59"/>
+      <c r="W10" s="53"/>
       <c r="X10" s="31">
         <v>20</v>
       </c>
@@ -2944,11 +2894,11 @@
       <c r="Q11" s="3">
         <v>10</v>
       </c>
-      <c r="S11" s="38"/>
+      <c r="S11" s="20"/>
       <c r="T11" s="18"/>
-      <c r="U11" s="59"/>
+      <c r="U11" s="53"/>
       <c r="V11" s="18"/>
-      <c r="W11" s="59"/>
+      <c r="W11" s="53"/>
       <c r="X11" s="31">
         <v>20</v>
       </c>
@@ -2996,11 +2946,11 @@
       <c r="Q12" s="3">
         <v>10</v>
       </c>
-      <c r="S12" s="38"/>
+      <c r="S12" s="20"/>
       <c r="T12" s="18"/>
-      <c r="U12" s="59"/>
+      <c r="U12" s="53"/>
       <c r="V12" s="18"/>
-      <c r="W12" s="59"/>
+      <c r="W12" s="53"/>
       <c r="X12" s="31">
         <v>20</v>
       </c>
@@ -3037,11 +2987,11 @@
       <c r="Q13" s="4">
         <v>5</v>
       </c>
-      <c r="S13" s="38"/>
+      <c r="S13" s="20"/>
       <c r="T13" s="18"/>
-      <c r="U13" s="59"/>
-      <c r="V13" s="59"/>
-      <c r="W13" s="59"/>
+      <c r="U13" s="53"/>
+      <c r="V13" s="53"/>
+      <c r="W13" s="53"/>
       <c r="X13" s="37">
         <v>20</v>
       </c>
@@ -3082,16 +3032,13 @@
       <c r="AC15" s="21"/>
       <c r="AD15" s="21"/>
     </row>
-    <row r="16" spans="4:30" ht="17.5" thickBot="1">
+    <row r="16" spans="4:30" ht="14.5" thickBot="1">
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
       <c r="F16" s="21"/>
-      <c r="H16" s="19" t="s">
-        <v>202</v>
-      </c>
       <c r="S16" s="20"/>
       <c r="W16" s="20"/>
-      <c r="X16" s="41" t="s">
+      <c r="X16" s="40" t="s">
         <v>132</v>
       </c>
       <c r="Y16" s="21"/>
@@ -3102,15 +3049,15 @@
       <c r="AD16" s="21"/>
     </row>
     <row r="17" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D17" s="38"/>
+      <c r="D17" s="20"/>
       <c r="E17" s="20"/>
       <c r="F17" s="20"/>
       <c r="G17" s="21"/>
-      <c r="S17" s="57"/>
-      <c r="T17" s="58"/>
-      <c r="U17" s="58"/>
-      <c r="V17" s="58"/>
-      <c r="W17" s="58"/>
+      <c r="S17" s="35"/>
+      <c r="T17" s="23"/>
+      <c r="U17" s="23"/>
+      <c r="V17" s="23"/>
+      <c r="W17" s="23"/>
       <c r="X17" s="22" t="s">
         <v>180</v>
       </c>
@@ -3129,28 +3076,28 @@
     </row>
     <row r="18" spans="4:30" ht="17.5" thickBot="1">
       <c r="D18" s="24" t="s">
+        <v>202</v>
+      </c>
+      <c r="E18" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="F18" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="G18" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="H18" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="H18" s="40" t="s">
+      <c r="I18" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="I18" s="22" t="s">
-        <v>208</v>
-      </c>
-      <c r="S18" s="38"/>
+      <c r="S18" s="20"/>
       <c r="T18" s="18"/>
-      <c r="U18" s="59"/>
+      <c r="U18" s="53"/>
       <c r="V18" s="18"/>
-      <c r="W18" s="59"/>
+      <c r="W18" s="53"/>
       <c r="X18" s="29">
         <v>10</v>
       </c>
@@ -3168,7 +3115,7 @@
       <c r="AD18" s="21"/>
     </row>
     <row r="19" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="40" t="s">
         <v>186</v>
       </c>
       <c r="E19" s="29">
@@ -3181,7 +3128,7 @@
         <f>SUM(N7+O7*(E19-1))</f>
         <v>610</v>
       </c>
-      <c r="H19" s="42">
+      <c r="H19" s="41">
         <f>SUM(P7+Q7*(E19-1))</f>
         <v>791</v>
       </c>
@@ -3189,11 +3136,11 @@
         <f>SUM(G19*((150+25*F19^2)/100))</f>
         <v>4727.5</v>
       </c>
-      <c r="S19" s="38"/>
+      <c r="S19" s="20"/>
       <c r="T19" s="18"/>
-      <c r="U19" s="59"/>
+      <c r="U19" s="53"/>
       <c r="V19" s="18"/>
-      <c r="W19" s="59"/>
+      <c r="W19" s="53"/>
       <c r="X19" s="31">
         <v>10</v>
       </c>
@@ -3211,7 +3158,7 @@
       <c r="AD19" s="21"/>
     </row>
     <row r="20" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="40" t="s">
         <v>189</v>
       </c>
       <c r="E20" s="29">
@@ -3221,10 +3168,10 @@
         <v>5</v>
       </c>
       <c r="G20" s="29">
-        <f>SUM(N8+O8*(E20-1))*0.75</f>
+        <f>SUM((N8+O8*(E20-1))*0.75)</f>
         <v>472.5</v>
       </c>
-      <c r="H20" s="42">
+      <c r="H20" s="41">
         <f t="shared" ref="H20:H25" si="0">SUM(P8+Q8*(E20-1))</f>
         <v>791</v>
       </c>
@@ -3234,11 +3181,11 @@
       </c>
       <c r="J20" s="21"/>
       <c r="K20" s="21"/>
-      <c r="S20" s="38"/>
+      <c r="S20" s="20"/>
       <c r="T20" s="18"/>
-      <c r="U20" s="59"/>
+      <c r="U20" s="53"/>
       <c r="V20" s="18"/>
-      <c r="W20" s="59"/>
+      <c r="W20" s="53"/>
       <c r="X20" s="31">
         <v>10</v>
       </c>
@@ -3256,7 +3203,7 @@
       <c r="AD20" s="21"/>
     </row>
     <row r="21" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="40" t="s">
         <v>192</v>
       </c>
       <c r="E21" s="29">
@@ -3269,7 +3216,7 @@
         <f>SUM(N9+O9*(E21-1))</f>
         <v>610</v>
       </c>
-      <c r="H21" s="42">
+      <c r="H21" s="41">
         <f t="shared" si="0"/>
         <v>791</v>
       </c>
@@ -3278,11 +3225,11 @@
         <v>2440</v>
       </c>
       <c r="J21" s="8"/>
-      <c r="S21" s="38"/>
+      <c r="S21" s="20"/>
       <c r="T21" s="18"/>
-      <c r="U21" s="59"/>
+      <c r="U21" s="53"/>
       <c r="V21" s="18"/>
-      <c r="W21" s="59"/>
+      <c r="W21" s="53"/>
       <c r="X21" s="31">
         <v>10</v>
       </c>
@@ -3300,7 +3247,7 @@
       <c r="AD21" s="21"/>
     </row>
     <row r="22" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="40" t="s">
         <v>194</v>
       </c>
       <c r="E22" s="29">
@@ -3313,7 +3260,7 @@
         <f>SUM(N10+O10*(E22-1)*0.75)</f>
         <v>472.5</v>
       </c>
-      <c r="H22" s="42">
+      <c r="H22" s="41">
         <f t="shared" si="0"/>
         <v>791</v>
       </c>
@@ -3322,11 +3269,11 @@
         <v>3071.25</v>
       </c>
       <c r="J22" s="8"/>
-      <c r="S22" s="38"/>
+      <c r="S22" s="20"/>
       <c r="T22" s="18"/>
-      <c r="U22" s="59"/>
+      <c r="U22" s="53"/>
       <c r="V22" s="18"/>
-      <c r="W22" s="59"/>
+      <c r="W22" s="53"/>
       <c r="X22" s="31">
         <v>10</v>
       </c>
@@ -3344,7 +3291,7 @@
       <c r="AD22" s="21"/>
     </row>
     <row r="23" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="40" t="s">
         <v>197</v>
       </c>
       <c r="E23" s="29">
@@ -3357,7 +3304,7 @@
         <f t="shared" ref="G23:G24" si="1">SUM(N11+O11*(E23-1))</f>
         <v>610</v>
       </c>
-      <c r="H23" s="42">
+      <c r="H23" s="41">
         <f t="shared" si="0"/>
         <v>791</v>
       </c>
@@ -3366,11 +3313,11 @@
         <v>3965</v>
       </c>
       <c r="J23" s="8"/>
-      <c r="S23" s="38"/>
+      <c r="S23" s="20"/>
       <c r="T23" s="18"/>
-      <c r="U23" s="59"/>
+      <c r="U23" s="53"/>
       <c r="V23" s="18"/>
-      <c r="W23" s="59"/>
+      <c r="W23" s="53"/>
       <c r="X23" s="31">
         <v>10</v>
       </c>
@@ -3388,7 +3335,7 @@
       <c r="AD23" s="21"/>
     </row>
     <row r="24" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="40" t="s">
         <v>200</v>
       </c>
       <c r="E24" s="29">
@@ -3401,7 +3348,7 @@
         <f t="shared" si="1"/>
         <v>610</v>
       </c>
-      <c r="H24" s="42">
+      <c r="H24" s="41">
         <f t="shared" si="0"/>
         <v>791</v>
       </c>
@@ -3410,11 +3357,11 @@
         <v>3965</v>
       </c>
       <c r="J24" s="8"/>
-      <c r="S24" s="38"/>
+      <c r="S24" s="20"/>
       <c r="T24" s="18"/>
-      <c r="U24" s="59"/>
-      <c r="V24" s="59"/>
-      <c r="W24" s="59"/>
+      <c r="U24" s="53"/>
+      <c r="V24" s="53"/>
+      <c r="W24" s="53"/>
       <c r="X24" s="37">
         <v>10</v>
       </c>
@@ -3432,24 +3379,24 @@
       <c r="AD24" s="21"/>
     </row>
     <row r="25" spans="4:30" ht="14.5" thickBot="1">
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="E25" s="43">
+      <c r="E25" s="42">
         <v>60</v>
       </c>
-      <c r="F25" s="43">
+      <c r="F25" s="42">
         <v>5</v>
       </c>
-      <c r="G25" s="43">
+      <c r="G25" s="42">
         <f>SUM(N13+O13*(E25-1))</f>
         <v>305</v>
       </c>
-      <c r="H25" s="43">
+      <c r="H25" s="42">
         <f t="shared" si="0"/>
         <v>395</v>
       </c>
-      <c r="I25" s="43">
+      <c r="I25" s="42">
         <f>SUM(G25*((150+50*F25)/100))</f>
         <v>1220</v>
       </c>
@@ -3487,7 +3434,7 @@
       <c r="AD27" s="21"/>
     </row>
     <row r="28" spans="4:30" ht="14.5" thickBot="1">
-      <c r="D28" s="38"/>
+      <c r="D28" s="20"/>
       <c r="E28" s="23"/>
       <c r="F28" s="23"/>
       <c r="G28" s="23"/>
@@ -3506,87 +3453,87 @@
       <c r="AD28" s="21"/>
     </row>
     <row r="29" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D29" s="38"/>
+      <c r="D29" s="20"/>
       <c r="E29" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="F29" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="F29" s="22" t="s">
+      <c r="G29" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="G29" s="22" t="s">
+      <c r="H29" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="H29" s="22" t="s">
-        <v>214</v>
-      </c>
-      <c r="I29" s="48" t="s">
+      <c r="I29" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="J29" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="J29" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="K29" s="62" t="s">
+      <c r="K29" s="56" t="s">
         <v>167</v>
       </c>
-      <c r="L29" s="63" t="s">
+      <c r="L29" s="57" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="30" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D30" s="41" t="s">
-        <v>209</v>
-      </c>
-      <c r="E30" s="56" t="s">
+      <c r="D30" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="E30" s="52" t="s">
         <v>164</v>
       </c>
       <c r="F30" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="G30" s="22" t="s">
         <v>215</v>
       </c>
-      <c r="G30" s="22" t="s">
-        <v>216</v>
-      </c>
-      <c r="H30" s="48" t="s">
+      <c r="H30" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="I30" s="55" t="s">
+      <c r="I30" s="51" t="s">
         <v>169</v>
       </c>
       <c r="J30" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="K30" s="62" t="s">
+        <v>214</v>
+      </c>
+      <c r="K30" s="56" t="s">
         <v>165</v>
       </c>
-      <c r="L30" s="53" t="s">
+      <c r="L30" s="49" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="31" spans="4:30" ht="17.5" thickBot="1">
-      <c r="D31" s="46" t="s">
-        <v>210</v>
-      </c>
-      <c r="E31" s="43">
-        <v>1</v>
-      </c>
-      <c r="F31" s="49" t="s">
+      <c r="D31" s="43" t="s">
+        <v>209</v>
+      </c>
+      <c r="E31" s="42">
+        <v>1</v>
+      </c>
+      <c r="F31" s="45" t="s">
         <v>168</v>
       </c>
-      <c r="G31" s="44" t="s">
+      <c r="G31" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="H31" s="44" t="s">
+      <c r="H31" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="I31" s="50">
-        <v>1</v>
-      </c>
-      <c r="J31" s="51" t="s">
+      <c r="I31" s="46">
+        <v>1</v>
+      </c>
+      <c r="J31" s="47" t="s">
         <v>168</v>
       </c>
-      <c r="K31" s="52" t="s">
+      <c r="K31" s="48" t="s">
         <v>168</v>
       </c>
-      <c r="L31" s="54" t="s">
+      <c r="L31" s="50" t="s">
         <v>168</v>
       </c>
     </row>
@@ -3597,22 +3544,22 @@
       <c r="E32" s="29" t="s">
         <v>168</v>
       </c>
-      <c r="F32" s="43">
+      <c r="F32" s="42">
         <f>SUM(G19+X7+(Z7*(E31-1)))</f>
         <v>630</v>
       </c>
-      <c r="G32" s="43">
+      <c r="G32" s="42">
         <f>SUM(H19+Y7+Z7*(E31-1))</f>
         <v>891</v>
       </c>
-      <c r="H32" s="43">
+      <c r="H32" s="42">
         <f>SUM(F32*((150+25*F19^2)/100))</f>
         <v>4882.5</v>
       </c>
-      <c r="I32" s="47" t="s">
+      <c r="I32" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="J32" s="54">
+      <c r="J32" s="50">
         <f>SUM(G19+X18+(Z18*(E31-1)))</f>
         <v>620</v>
       </c>
@@ -3620,9 +3567,9 @@
         <f>SUM(H19+Y18+AA18*(I31-1))</f>
         <v>841</v>
       </c>
-      <c r="L32" s="43">
-        <f>SUM(J32*((150+25*J19^2)/100))</f>
-        <v>930</v>
+      <c r="L32" s="42">
+        <f>SUM(J32*((150+25*F20^2)/100))</f>
+        <v>4805</v>
       </c>
     </row>
     <row r="33" spans="4:12" ht="17.5" thickBot="1">
@@ -3632,22 +3579,22 @@
       <c r="E33" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="F33" s="43">
+      <c r="F33" s="42">
         <f>SUM(G20+X8+(Z8*(E31-1)))</f>
         <v>492.5</v>
       </c>
-      <c r="G33" s="43">
+      <c r="G33" s="42">
         <f>SUM(H20+Y8+Z8*(E31-1))</f>
         <v>891</v>
       </c>
-      <c r="H33" s="43">
+      <c r="H33" s="42">
         <f>SUM(F33*((120+20*F20)/100))</f>
         <v>1083.5</v>
       </c>
-      <c r="I33" s="47" t="s">
+      <c r="I33" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="J33" s="54">
+      <c r="J33" s="50">
         <f>SUM(G20+X19+(Z19*(E31-1)))</f>
         <v>482.5</v>
       </c>
@@ -3655,9 +3602,9 @@
         <f>SUM(H20+Y19+AA19*(I31-1))</f>
         <v>841</v>
       </c>
-      <c r="L33" s="43">
-        <f>SUM(J33*((120+20*J20)/100))</f>
-        <v>579</v>
+      <c r="L33" s="42">
+        <f>SUM(J33*((120+20*F20)/100))</f>
+        <v>1061.5</v>
       </c>
     </row>
     <row r="34" spans="4:12" ht="17.5" thickBot="1">
@@ -3667,22 +3614,22 @@
       <c r="E34" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="F34" s="43">
+      <c r="F34" s="42">
         <f>SUM(G21+X9+(Z9*(E31-1)))</f>
         <v>630</v>
       </c>
-      <c r="G34" s="43">
+      <c r="G34" s="42">
         <f>SUM(H21+Y9+Z9*(E31-1))</f>
         <v>891</v>
       </c>
-      <c r="H34" s="43">
+      <c r="H34" s="42">
         <f>SUM(F34*((150+50*F21)/100))</f>
         <v>2520</v>
       </c>
-      <c r="I34" s="47" t="s">
+      <c r="I34" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="J34" s="54">
+      <c r="J34" s="50">
         <f>SUM(G21+X20+(Z20*(E31-1)))</f>
         <v>620</v>
       </c>
@@ -3690,9 +3637,9 @@
         <f>SUM(H21+Y20+AA20*(I31-1))</f>
         <v>841</v>
       </c>
-      <c r="L34" s="43">
-        <f>SUM(J34*((150+50*J21)/100))</f>
-        <v>930</v>
+      <c r="L34" s="42">
+        <f>SUM(J34*((150+50*F21)/100))</f>
+        <v>2480</v>
       </c>
     </row>
     <row r="35" spans="4:12" ht="17.5" thickBot="1">
@@ -3702,22 +3649,22 @@
       <c r="E35" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="F35" s="43">
+      <c r="F35" s="42">
         <f>SUM(G22+X10+(Z10*(E31-1)))</f>
         <v>492.5</v>
       </c>
-      <c r="G35" s="43">
+      <c r="G35" s="42">
         <f>SUM(H22+Y10+Z10*(E31-1))</f>
         <v>891</v>
       </c>
-      <c r="H35" s="43">
+      <c r="H35" s="42">
         <f>SUM(F35*((12.5*F22^2+37.5*F22+150)/100))</f>
         <v>3201.25</v>
       </c>
-      <c r="I35" s="47" t="s">
+      <c r="I35" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="J35" s="54">
+      <c r="J35" s="50">
         <f>SUM(G22+X21+(Z21*(E31-1)))</f>
         <v>482.5</v>
       </c>
@@ -3725,9 +3672,9 @@
         <f>SUM(H22+Y21+AA21*(I31-1))</f>
         <v>841</v>
       </c>
-      <c r="L35" s="43">
-        <f>SUM(J35*((12.5*J22^2+37.5*J22+150)/100))</f>
-        <v>723.75</v>
+      <c r="L35" s="42">
+        <f>SUM(J35*((12.5*F22^2+37.5*F22+150)/100))</f>
+        <v>3136.25</v>
       </c>
     </row>
     <row r="36" spans="4:12" ht="17.5" thickBot="1">
@@ -3737,22 +3684,22 @@
       <c r="E36" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="F36" s="43">
+      <c r="F36" s="42">
         <f>SUM(G23+X11+(Z11*(E31-1)))</f>
         <v>630</v>
       </c>
-      <c r="G36" s="43">
+      <c r="G36" s="42">
         <f>SUM(H23+Y11+Z11*(E31-1))</f>
         <v>891</v>
       </c>
-      <c r="H36" s="43">
+      <c r="H36" s="42">
         <f>SUM(F36*((12.5*F23^2+37.5*F23+150)/100))</f>
         <v>4095</v>
       </c>
-      <c r="I36" s="47" t="s">
+      <c r="I36" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="J36" s="54">
+      <c r="J36" s="50">
         <f>SUM(G23+X22+(Z22*(E31-1)))</f>
         <v>620</v>
       </c>
@@ -3760,9 +3707,9 @@
         <f>SUM(H23+Y22+AA22*(I31-1))</f>
         <v>841</v>
       </c>
-      <c r="L36" s="43">
-        <f>SUM(J36*((12.5*J23^2+37.5*J23+150)/100))</f>
-        <v>930</v>
+      <c r="L36" s="42">
+        <f>SUM(J36*((12.5*F23^2+37.5*F23+150)/100))</f>
+        <v>4030</v>
       </c>
     </row>
     <row r="37" spans="4:12" ht="17.5" thickBot="1">
@@ -3772,22 +3719,22 @@
       <c r="E37" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="F37" s="43">
+      <c r="F37" s="42">
         <f>SUM(G24+X12+(Z12*(E31-1)))</f>
         <v>630</v>
       </c>
-      <c r="G37" s="43">
+      <c r="G37" s="42">
         <f>SUM(H24+Y12+Z12*(E31-1))</f>
         <v>891</v>
       </c>
-      <c r="H37" s="43">
+      <c r="H37" s="42">
         <f>SUM(F37*((12.5*F24^2+37.5*F24+150)/100))</f>
         <v>4095</v>
       </c>
-      <c r="I37" s="47" t="s">
+      <c r="I37" s="44" t="s">
         <v>168</v>
       </c>
-      <c r="J37" s="54">
+      <c r="J37" s="50">
         <f>SUM(G24+X23+(Z23*(E31-1)))</f>
         <v>620</v>
       </c>
@@ -3795,9 +3742,9 @@
         <f>SUM(H24+Y23+AA23*(I31-1))</f>
         <v>841</v>
       </c>
-      <c r="L37" s="43">
-        <f>SUM(J37*((12.5*J24^2+37.5*J24+150)/100))</f>
-        <v>930</v>
+      <c r="L37" s="42">
+        <f>SUM(J37*((12.5*F24^2+37.5*F24+150)/100))</f>
+        <v>4030</v>
       </c>
     </row>
     <row r="38" spans="4:12" ht="14.5" thickBot="1">
@@ -3807,68 +3754,64 @@
       <c r="E38" s="37" t="s">
         <v>168</v>
       </c>
-      <c r="F38" s="43">
+      <c r="F38" s="42">
         <f>SUM(G25+X13+(Z13*(E31-1)))</f>
         <v>325</v>
       </c>
-      <c r="G38" s="43">
+      <c r="G38" s="42">
         <f>SUM(H25+Y13+Z13*(E31-1))</f>
         <v>495</v>
       </c>
-      <c r="H38" s="43">
+      <c r="H38" s="42">
         <f>SUM(F38*((150+50*F25)/100))</f>
         <v>1300</v>
       </c>
       <c r="I38" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="J38" s="54">
+      <c r="J38" s="50">
         <f>SUM(G25+X24+(Z24*(E31-1)))</f>
         <v>315</v>
       </c>
-      <c r="K38" s="43">
+      <c r="K38" s="42">
         <f>SUM(H25+Y24+AA24*(I31-1))</f>
         <v>445</v>
       </c>
-      <c r="L38" s="43">
-        <f>SUM(J38*((150+50*J25)/100))</f>
-        <v>472.5</v>
+      <c r="L38" s="42">
+        <f>SUM(J38*((150+50*F25)/100))</f>
+        <v>1260</v>
       </c>
     </row>
     <row r="39" spans="4:12">
       <c r="D39" s="20"/>
-      <c r="E39" s="44"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="45"/>
-      <c r="I39" s="45"/>
+      <c r="E39" s="21"/>
     </row>
     <row r="40" spans="4:12">
       <c r="D40" s="20"/>
       <c r="E40" s="20"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="45"/>
     </row>
     <row r="41" spans="4:12">
       <c r="D41" s="20"/>
       <c r="E41" s="20"/>
-      <c r="F41" s="45"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="45"/>
-      <c r="I41" s="45"/>
-    </row>
-    <row r="42" spans="4:12">
-      <c r="F42" s="45"/>
-      <c r="G42" s="45"/>
-      <c r="H42" s="45"/>
-      <c r="I42" s="45"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="F32:F38">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF555A"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{6DC8F541-8D43-4756-ACEC-41C261A67E6C}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G19:G25">
-    <cfRule type="dataBar" priority="15">
+    <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3881,8 +3824,22 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G32:G38">
+    <cfRule type="dataBar" priority="5">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{547E64C2-EEE7-432F-86C2-527CD3952354}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H19:H25">
-    <cfRule type="dataBar" priority="1">
+    <cfRule type="dataBar" priority="6">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3895,36 +3852,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I19:I25">
-    <cfRule type="dataBar" priority="16">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF63C384"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F2C7C6CE-E2BB-4479-A10D-20BDEAF834BF}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G32:G38">
-    <cfRule type="dataBar" priority="6">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF008AEF"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{547E64C2-EEE7-432F-86C2-527CD3952354}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H32">
-    <cfRule type="dataBar" priority="13">
+    <cfRule type="dataBar" priority="22">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3938,7 +3867,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H33">
-    <cfRule type="dataBar" priority="12">
+    <cfRule type="dataBar" priority="21">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3952,7 +3881,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H34:H38">
-    <cfRule type="dataBar" priority="11">
+    <cfRule type="dataBar" priority="20">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3965,8 +3894,36 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I19:I25">
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F2C7C6CE-E2BB-4479-A10D-20BDEAF834BF}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J32:J38">
+    <cfRule type="dataBar" priority="3">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF555A"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BAFF5A6F-A007-475F-B2B1-9B8F81ACCC24}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K32:K38">
-    <cfRule type="dataBar" priority="2">
+    <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3979,36 +3936,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J32:J38">
-    <cfRule type="dataBar" priority="9">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFF555A"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BAFF5A6F-A007-475F-B2B1-9B8F81ACCC24}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F32:F38">
-    <cfRule type="dataBar" priority="7">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFF555A"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6DC8F541-8D43-4756-ACEC-41C261A67E6C}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="L32">
-    <cfRule type="dataBar" priority="5">
+    <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4022,7 +3951,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L33">
-    <cfRule type="dataBar" priority="4">
+    <cfRule type="dataBar" priority="13">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4036,7 +3965,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L34:L38">
-    <cfRule type="dataBar" priority="3">
+    <cfRule type="dataBar" priority="12">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -4049,10 +3978,51 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L32:L38">
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F374C5A9-D849-4819-9E5E-AD66F9B97C0B}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32:H38">
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{077659C4-813B-4775-84AF-3BC0A328CF66}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{6DC8F541-8D43-4756-ACEC-41C261A67E6C}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFF555A"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>F32:F38</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{F9FF934E-07C0-4A27-9A29-453DAA51FCCB}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
@@ -4067,6 +4037,19 @@
           <xm:sqref>G19:G25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{547E64C2-EEE7-432F-86C2-527CD3952354}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G32:G38</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{EF1B277A-C5C5-4416-BA7D-7E93D6CD9AE9}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -4078,32 +4061,6 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>H19:H25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F2C7C6CE-E2BB-4479-A10D-20BDEAF834BF}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF63C384"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>I19:I25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{547E64C2-EEE7-432F-86C2-527CD3952354}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>G32:G38</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C2CB533B-EA72-4E80-AAF4-3437086B381B}">
@@ -4145,17 +4102,17 @@
           <xm:sqref>H34:H38</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{794CA5F0-0896-408D-90FD-672497C8543F}">
+          <x14:cfRule type="dataBar" id="{F2C7C6CE-E2BB-4479-A10D-20BDEAF834BF}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FF008AEF"/>
+              <x14:borderColor rgb="FF63C384"/>
               <x14:negativeFillColor rgb="FFFF0000"/>
               <x14:negativeBorderColor rgb="FFFF0000"/>
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>K32:K38</xm:sqref>
+          <xm:sqref>I19:I25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{BAFF5A6F-A007-475F-B2B1-9B8F81ACCC24}">
@@ -4171,17 +4128,17 @@
           <xm:sqref>J32:J38</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6DC8F541-8D43-4756-ACEC-41C261A67E6C}">
+          <x14:cfRule type="dataBar" id="{794CA5F0-0896-408D-90FD-672497C8543F}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFF555A"/>
+              <x14:borderColor rgb="FF008AEF"/>
               <x14:negativeFillColor rgb="FFFF0000"/>
               <x14:negativeBorderColor rgb="FFFF0000"/>
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>F32:F38</xm:sqref>
+          <xm:sqref>K32:K38</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{64D70BFC-6F3C-4D88-A753-C42A0873A464}">
@@ -4221,6 +4178,32 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>L34:L38</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F374C5A9-D849-4819-9E5E-AD66F9B97C0B}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>L32:L38</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{077659C4-813B-4775-84AF-3BC0A328CF66}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>H32:H38</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>